<commit_message>
updates to excel files for wildfire runs
</commit_message>
<xml_diff>
--- a/cache/Wildfire/wildfire_runs.xlsx
+++ b/cache/Wildfire/wildfire_runs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnnickDewald\PycharmProjects\DawnDesignTool\cache\Wildfire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCA79CB-78E9-4B30-BC59-F2A289F5A06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E26E0D-AA4D-43AB-86FD-B02DCFCB0B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" xr2:uid="{5B225A7C-2425-4B12-971A-E195856C5D49}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{5B225A7C-2425-4B12-971A-E195856C5D49}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="27">
   <si>
     <t>battery_specific_energy_Wh_kg</t>
   </si>
   <si>
-    <t>solar_cell_efficiency</t>
-  </si>
-  <si>
     <t xml:space="preserve">run_num </t>
   </si>
   <si>
@@ -59,64 +56,67 @@
     <t>no</t>
   </si>
   <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 331.5 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
     <t>required_snr</t>
   </si>
   <si>
-    <t>revisit_rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coverage_radius </t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 5m resolution, 331.5 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
     <t>spatial_resolution</t>
   </si>
   <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 382.5 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 100m resolution, 331.5 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 100m resolution, 382.5 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
     <t>structural_mass_margin_multiplier</t>
   </si>
   <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 405 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 450 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 495 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 540 Wh/kg battery pack, 26% solar efficiency</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 2km radius coverage area, revisit every 12 hours, 25% struct. margin</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 2km radius coverage area, revisit every 12 hours, 10% struct. margin</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 2km radius coverage area, revisit every 12 hours, 5% struct. margin</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 2km radius coverage area, revisit every 12 hours, 15% struct. margin</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 2km radius coverage area, revisit every 6 hours, 25% struct. margin</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 450 Wh/kg battery pack, 30% solar efficiency</t>
+    <t>solar_cell_efficiency_cell_level</t>
+  </si>
+  <si>
+    <t>required_spatial_coverage</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 4180km^2 spatial coverage, revisit every 12 hours, 10% struct. margin</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 5m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 5m resolution, 450 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 100m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 4180km^2 spatial coverage, revisit every 6 hours, 10% struct. margin</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 100m resolution, 450 Wh/kg battery cell, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 390 Wh/kg battery cell, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 500 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 550 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 100m resolution, 600 Wh/kg battery cell, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 1860km^2 spatial coverage, revisit every 12 hours, 10% struct. margin</t>
+  </si>
+  <si>
+    <t>required_revisit_rate</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 1m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
   </si>
 </sst>
 </file>
@@ -468,52 +468,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEA4D99-B955-4859-B9C9-8BD4545DD517}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" customWidth="1"/>
     <col min="2" max="2" width="31.109375" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" customWidth="1"/>
     <col min="4" max="4" width="10.88671875" customWidth="1"/>
     <col min="5" max="7" width="16.109375" customWidth="1"/>
     <col min="10" max="10" width="75.44140625" customWidth="1"/>
-    <col min="11" max="11" width="89.6640625" customWidth="1"/>
+    <col min="11" max="11" width="95.88671875" customWidth="1"/>
     <col min="12" max="12" width="76.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>4</v>
-      </c>
-      <c r="K1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -524,31 +524,31 @@
         <v>390</v>
       </c>
       <c r="C2">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D2">
         <v>2</v>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -559,31 +559,31 @@
         <v>390</v>
       </c>
       <c r="C3">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -594,31 +594,31 @@
         <v>450</v>
       </c>
       <c r="C4">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D4">
         <v>2</v>
       </c>
       <c r="E4">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
       <c r="G4">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -629,31 +629,31 @@
         <v>390</v>
       </c>
       <c r="C5">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
       <c r="E5">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F5">
         <v>100</v>
       </c>
       <c r="G5">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H5">
         <v>3</v>
       </c>
       <c r="I5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -664,31 +664,31 @@
         <v>390</v>
       </c>
       <c r="C6">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D6">
         <v>4</v>
       </c>
       <c r="E6">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F6">
         <v>5</v>
       </c>
       <c r="G6">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H6">
         <v>4</v>
       </c>
       <c r="I6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K6" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -699,31 +699,31 @@
         <v>450</v>
       </c>
       <c r="C7">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F7">
         <v>100</v>
       </c>
       <c r="G7">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H7">
         <v>5</v>
       </c>
       <c r="I7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K7" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -731,7 +731,7 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>500</v>
+        <v>390</v>
       </c>
       <c r="C8">
         <v>0.3</v>
@@ -740,25 +740,25 @@
         <v>2</v>
       </c>
       <c r="E8">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F8">
         <v>5</v>
       </c>
       <c r="G8">
-        <v>1.25</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H8">
         <v>6</v>
       </c>
       <c r="I8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="K8" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -766,16 +766,16 @@
         <v>20</v>
       </c>
       <c r="B9">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C9">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D9">
         <v>2</v>
       </c>
       <c r="E9">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -787,13 +787,13 @@
         <v>7</v>
       </c>
       <c r="I9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K9" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -801,16 +801,16 @@
         <v>20</v>
       </c>
       <c r="B10">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="C10">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
       <c r="E10">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F10">
         <v>5</v>
@@ -822,13 +822,13 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -836,16 +836,16 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <v>550</v>
+        <v>600</v>
       </c>
       <c r="C11">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -857,13 +857,13 @@
         <v>9</v>
       </c>
       <c r="I11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K11" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -874,13 +874,13 @@
         <v>600</v>
       </c>
       <c r="C12">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
       <c r="E12">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F12">
         <v>5</v>
@@ -892,48 +892,48 @@
         <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K12" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B13">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="C13">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
       <c r="E13">
-        <v>2000</v>
+        <v>4178000000</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="G13">
-        <v>1.05</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H13">
         <v>11</v>
       </c>
       <c r="I13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J13" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="K13" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -941,37 +941,73 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>450</v>
+        <v>390</v>
       </c>
       <c r="C14">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D14">
         <v>2</v>
       </c>
       <c r="E14">
-        <v>2000</v>
+        <v>1858000000</v>
       </c>
       <c r="F14">
         <v>5</v>
       </c>
       <c r="G14">
-        <v>1.1499999999999999</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H14">
         <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J14" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K14" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>390</v>
+      </c>
+      <c r="C15">
+        <v>0.25</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15">
+        <v>4178000000</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H15">
+        <v>13</v>
+      </c>
+      <c r="I15" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updates to run specs  and title label files
</commit_message>
<xml_diff>
--- a/cache/Wildfire/wildfire_runs.xlsx
+++ b/cache/Wildfire/wildfire_runs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnnickDewald\PycharmProjects\DawnDesignTool\cache\Wildfire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E26E0D-AA4D-43AB-86FD-B02DCFCB0B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346DB6FB-1CBA-43DA-A058-48ABE3995C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{5B225A7C-2425-4B12-971A-E195856C5D49}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5B225A7C-2425-4B12-971A-E195856C5D49}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,52 +71,52 @@
     <t>required_spatial_coverage</t>
   </si>
   <si>
-    <t>min alt set by strat height, no alt. cycling, 4180km^2 spatial coverage, revisit every 12 hours, 10% struct. margin</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 5m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 5m resolution, 450 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 100m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 4180km^2 spatial coverage, revisit every 6 hours, 10% struct. margin</t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 100m resolution, 450 Wh/kg battery cell, 30% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 390 Wh/kg battery cell, 30% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 500 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 550 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell, 25% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell, 30% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>SAR Payload, 6 dB SNR, 100m resolution, 600 Wh/kg battery cell, 30% solar cell efficiency</t>
-  </si>
-  <si>
-    <t>min alt set by strat height, no alt. cycling, 1860km^2 spatial coverage, revisit every 12 hours, 10% struct. margin</t>
-  </si>
-  <si>
     <t>required_revisit_rate</t>
   </si>
   <si>
-    <t>SAR Payload, 20 dB SNR, 1m resolution, 390 Wh/kg battery cell, 25% solar cell efficiency</t>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 390 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 100m resolution, 450 Wh/kg battery cell energy density, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 500 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 550 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 600 Wh/kg battery cell energy density, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 100m resolution, 600 Wh/kg battery cell energy density, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 450 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 6 dB SNR, 5m resolution, 450 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 100m resolution, 450 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 5m resolution, 450 Wh/kg battery cell energy density, 30% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>SAR Payload, 20 dB SNR, 1m resolution, 450 Wh/kg battery cell energy density, 25% solar cell efficiency</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 5000km^2 spatial coverage, revisit rate 2/day, 10% struct. margin</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 5000km^2 spatial coverage, revisit rate 4/day, 10% struct. margin</t>
+  </si>
+  <si>
+    <t>min alt set by strat height, no alt. cycling, 2500km^2 spatial coverage, revisit rate 2/day, 10% struct. margin</t>
   </si>
 </sst>
 </file>
@@ -492,7 +492,7 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
@@ -521,7 +521,7 @@
         <v>20</v>
       </c>
       <c r="B2">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C2">
         <v>0.25</v>
@@ -530,7 +530,7 @@
         <v>2</v>
       </c>
       <c r="E2">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -545,10 +545,10 @@
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -556,7 +556,7 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C3">
         <v>0.25</v>
@@ -565,7 +565,7 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -580,10 +580,10 @@
         <v>5</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -591,7 +591,7 @@
         <v>20</v>
       </c>
       <c r="B4">
-        <v>450</v>
+        <v>390</v>
       </c>
       <c r="C4">
         <v>0.25</v>
@@ -600,7 +600,7 @@
         <v>2</v>
       </c>
       <c r="E4">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F4">
         <v>5</v>
@@ -615,10 +615,10 @@
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -626,7 +626,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C5">
         <v>0.25</v>
@@ -635,7 +635,7 @@
         <v>2</v>
       </c>
       <c r="E5">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F5">
         <v>100</v>
@@ -650,10 +650,10 @@
         <v>5</v>
       </c>
       <c r="J5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K5" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -661,7 +661,7 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C6">
         <v>0.25</v>
@@ -670,7 +670,7 @@
         <v>4</v>
       </c>
       <c r="E6">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -685,10 +685,10 @@
         <v>5</v>
       </c>
       <c r="J6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="K6" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -705,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F7">
         <v>100</v>
@@ -720,10 +720,10 @@
         <v>5</v>
       </c>
       <c r="J7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K7" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -731,7 +731,7 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C8">
         <v>0.3</v>
@@ -740,7 +740,7 @@
         <v>2</v>
       </c>
       <c r="E8">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -755,10 +755,10 @@
         <v>5</v>
       </c>
       <c r="J8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -775,7 +775,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F9">
         <v>5</v>
@@ -790,10 +790,10 @@
         <v>5</v>
       </c>
       <c r="J9" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K9" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -810,7 +810,7 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F10">
         <v>5</v>
@@ -825,10 +825,10 @@
         <v>5</v>
       </c>
       <c r="J10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K10" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
@@ -845,7 +845,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -860,10 +860,10 @@
         <v>5</v>
       </c>
       <c r="J11" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K11" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
@@ -880,7 +880,7 @@
         <v>2</v>
       </c>
       <c r="E12">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F12">
         <v>5</v>
@@ -895,10 +895,10 @@
         <v>5</v>
       </c>
       <c r="J12" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K12" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -915,7 +915,7 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F13">
         <v>100</v>
@@ -930,10 +930,10 @@
         <v>5</v>
       </c>
       <c r="J13" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K13" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
@@ -941,7 +941,7 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C14">
         <v>0.25</v>
@@ -950,7 +950,7 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <v>1858000000</v>
+        <v>2500000000</v>
       </c>
       <c r="F14">
         <v>5</v>
@@ -965,10 +965,10 @@
         <v>5</v>
       </c>
       <c r="J14" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="K14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -976,7 +976,7 @@
         <v>20</v>
       </c>
       <c r="B15">
-        <v>390</v>
+        <v>450</v>
       </c>
       <c r="C15">
         <v>0.25</v>
@@ -985,7 +985,7 @@
         <v>2</v>
       </c>
       <c r="E15">
-        <v>4178000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1000,10 +1000,10 @@
         <v>5</v>
       </c>
       <c r="J15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="K15" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>